<commit_message>
chore: Regenerate production output with R.2B EngineeringContext consumption
Updated Estimation_Output.xlsx and JSON artefacts after Fe550/30mm cover/50d Ld
parameters from GN DXF. Total steel weight: 615.9 kg.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Version7/data/output/Production_Output/Engineering_Review.xlsx
+++ b/Version7/data/output/Production_Output/Engineering_Review.xlsx
@@ -609,7 +609,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Galera Estimation — Benchmark Set 1</t>
+          <t>Galera Estimation — Benchmark Set 2</t>
         </is>
       </c>
     </row>
@@ -621,7 +621,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>C25/30</t>
+          <t>M30</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Fe415 (High Yield)</t>
+          <t>Fe550 (High Yield)</t>
         </is>
       </c>
     </row>
@@ -645,7 +645,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>30</t>
         </is>
       </c>
     </row>
@@ -657,7 +657,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>V6.6.0 Production Output Engine</t>
+          <t>V7.6.0 Production Output Engine (R.2B)</t>
         </is>
       </c>
     </row>
@@ -681,7 +681,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>2026-07-15 12:18:56</t>
+          <t>2026-07-15 18:27:03</t>
         </is>
       </c>
     </row>
@@ -722,28 +722,28 @@
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>2. Development length = 40d (IS 456:2000, Fe415, M25).</t>
+          <t>2. Development length from GN DXF table (Fe550, M30) — factor ~50d for dia=12.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>3. Stirrup hook allowance = 2 x 10d (135-degree hook).</t>
+          <t>3. Stirrup hook allowance = 2 x 5d (135-degree hook, from GN DXF).</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>4. Clear cover = 40 mm (IS 456:2000 Table 16).</t>
+          <t>4. Clear cover = 30 mm (from GN DXF TABLE 2).</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>5. Steel density = 7850 kg/m³.</t>
+          <t>5. Steel density = 7850.0 kg/m³.</t>
         </is>
       </c>
     </row>
@@ -757,28 +757,28 @@
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>7. Stirrup cut length = 2(W-2c) + 2(D-2c) + 2x10d.</t>
+          <t>7. Stirrup cut length = 2(W-2c) + 2(D-2c) + 2x5d.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>8. Y = High Yield Deformed bars (Fe415).</t>
+          <t>8. Y = High Yield Deformed bars (Fe550).</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>9. This schedule is for engineering review and manual verification.</t>
+          <t>9. Minimum lap splice = 300 mm (from GN DXF).</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>10. Phase V.B.1 — Production Output Completion (MODEL_VERSION 6.6.0).</t>
+          <t>10. Phase R.2B — Engineering Context Consumption (MODEL_VERSION 7.6.0).</t>
         </is>
       </c>
     </row>
@@ -917,22 +917,22 @@
         <v>10</v>
       </c>
       <c r="F3" s="7" t="n">
-        <v>208.99</v>
+        <v>216.042</v>
       </c>
       <c r="G3" s="7" t="n">
-        <v>4.901</v>
+        <v>5.027</v>
       </c>
       <c r="H3" s="7" t="n">
-        <v>51.099</v>
+        <v>50.408</v>
       </c>
       <c r="I3" s="7" t="n">
-        <v>17.392</v>
+        <v>18.032</v>
       </c>
       <c r="J3" s="7" t="n">
-        <v>64.87</v>
+        <v>67.90000000000001</v>
       </c>
       <c r="K3" s="7" t="n">
-        <v>70.729</v>
+        <v>74.675</v>
       </c>
       <c r="L3" s="7" t="n">
         <v>0</v>
@@ -960,19 +960,19 @@
         <v>10</v>
       </c>
       <c r="F4" s="9" t="n">
-        <v>109.146</v>
+        <v>114.165</v>
       </c>
       <c r="G4" s="9" t="n">
-        <v>26.319</v>
+        <v>26.445</v>
       </c>
       <c r="H4" s="9" t="n">
         <v>0</v>
       </c>
       <c r="I4" s="9" t="n">
-        <v>17.295</v>
+        <v>18.147</v>
       </c>
       <c r="J4" s="9" t="n">
-        <v>65.533</v>
+        <v>69.57299999999999</v>
       </c>
       <c r="K4" s="9" t="n">
         <v>0</v>
@@ -1393,7 +1393,7 @@
         <v>8</v>
       </c>
       <c r="F15" s="7" t="n">
-        <v>109.816</v>
+        <v>115.578</v>
       </c>
       <c r="G15" s="7" t="n">
         <v>20.455</v>
@@ -1402,16 +1402,16 @@
         <v>0</v>
       </c>
       <c r="I15" s="7" t="n">
-        <v>18.609</v>
+        <v>19.461</v>
       </c>
       <c r="J15" s="7" t="n">
-        <v>17.551</v>
+        <v>18.561</v>
       </c>
       <c r="K15" s="7" t="n">
-        <v>29.002</v>
+        <v>30.975</v>
       </c>
       <c r="L15" s="7" t="n">
-        <v>24.199</v>
+        <v>26.126</v>
       </c>
       <c r="M15" s="7" t="n">
         <v>0</v>
@@ -3347,19 +3347,19 @@
         <v>10</v>
       </c>
       <c r="F65" s="7" t="n">
-        <v>71.151</v>
+        <v>76.17100000000001</v>
       </c>
       <c r="G65" s="7" t="n">
-        <v>15.341</v>
+        <v>15.468</v>
       </c>
       <c r="H65" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I65" s="7" t="n">
-        <v>11.364</v>
+        <v>12.216</v>
       </c>
       <c r="J65" s="7" t="n">
-        <v>44.446</v>
+        <v>48.486</v>
       </c>
       <c r="K65" s="7" t="n">
         <v>0</v>
@@ -3390,19 +3390,19 @@
         <v>10</v>
       </c>
       <c r="F66" s="9" t="n">
-        <v>88.931</v>
+        <v>93.95</v>
       </c>
       <c r="G66" s="9" t="n">
-        <v>20.503</v>
+        <v>20.629</v>
       </c>
       <c r="H66" s="9" t="n">
         <v>0</v>
       </c>
       <c r="I66" s="9" t="n">
-        <v>14.134</v>
+        <v>14.986</v>
       </c>
       <c r="J66" s="9" t="n">
-        <v>54.295</v>
+        <v>58.335</v>
       </c>
       <c r="K66" s="9" t="n">
         <v>0</v>
@@ -3466,25 +3466,25 @@
         <v>65</v>
       </c>
       <c r="F68" s="11" t="n">
-        <v>588.035</v>
+        <v>615.9059999999999</v>
       </c>
       <c r="G68" s="11" t="n">
-        <v>87.51900000000001</v>
+        <v>88.024</v>
       </c>
       <c r="H68" s="11" t="n">
-        <v>51.099</v>
+        <v>50.408</v>
       </c>
       <c r="I68" s="11" t="n">
-        <v>78.79300000000001</v>
+        <v>82.842</v>
       </c>
       <c r="J68" s="11" t="n">
-        <v>246.694</v>
+        <v>262.856</v>
       </c>
       <c r="K68" s="11" t="n">
-        <v>99.73099999999999</v>
+        <v>105.65</v>
       </c>
       <c r="L68" s="11" t="n">
-        <v>24.199</v>
+        <v>26.126</v>
       </c>
       <c r="M68" s="11" t="n">
         <v>0</v>
@@ -3656,7 +3656,7 @@
       <c r="O3" s="12" t="n"/>
       <c r="P3" s="12" t="n"/>
       <c r="Q3" s="12" t="n">
-        <v>208.9904488910203</v>
+        <v>216.0416656374083</v>
       </c>
     </row>
     <row r="4">
@@ -3679,25 +3679,25 @@
         <v>2</v>
       </c>
       <c r="G4" s="7" t="n">
-        <v>1.28</v>
+        <v>1.6</v>
       </c>
       <c r="H4" s="7" t="n">
-        <v>6.85</v>
+        <v>7.17</v>
       </c>
       <c r="I4" s="7" t="n">
-        <v>13.7</v>
+        <v>14.34</v>
       </c>
       <c r="J4" s="6" t="n"/>
       <c r="K4" s="6" t="n"/>
       <c r="L4" s="6" t="n"/>
       <c r="M4" s="7" t="n">
-        <v>21.623</v>
+        <v>22.633</v>
       </c>
       <c r="N4" s="6" t="n"/>
       <c r="O4" s="6" t="n"/>
       <c r="P4" s="6" t="n"/>
       <c r="Q4" s="7" t="n">
-        <v>21.623</v>
+        <v>22.633</v>
       </c>
     </row>
     <row r="5">
@@ -3720,25 +3720,25 @@
         <v>2</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>1.28</v>
+        <v>1.6</v>
       </c>
       <c r="H5" s="9" t="n">
-        <v>6.85</v>
+        <v>7.17</v>
       </c>
       <c r="I5" s="9" t="n">
-        <v>13.7</v>
+        <v>14.34</v>
       </c>
       <c r="J5" s="8" t="n"/>
       <c r="K5" s="8" t="n"/>
       <c r="L5" s="8" t="n"/>
       <c r="M5" s="9" t="n">
-        <v>21.623</v>
+        <v>22.633</v>
       </c>
       <c r="N5" s="8" t="n"/>
       <c r="O5" s="8" t="n"/>
       <c r="P5" s="8" t="n"/>
       <c r="Q5" s="9" t="n">
-        <v>21.623</v>
+        <v>22.633</v>
       </c>
     </row>
     <row r="6">
@@ -3761,25 +3761,25 @@
         <v>2</v>
       </c>
       <c r="G6" s="7" t="n">
-        <v>1.28</v>
+        <v>1.6</v>
       </c>
       <c r="H6" s="7" t="n">
-        <v>6.85</v>
+        <v>7.17</v>
       </c>
       <c r="I6" s="7" t="n">
-        <v>13.7</v>
+        <v>14.34</v>
       </c>
       <c r="J6" s="6" t="n"/>
       <c r="K6" s="6" t="n"/>
       <c r="L6" s="6" t="n"/>
       <c r="M6" s="7" t="n">
-        <v>21.623</v>
+        <v>22.633</v>
       </c>
       <c r="N6" s="6" t="n"/>
       <c r="O6" s="6" t="n"/>
       <c r="P6" s="6" t="n"/>
       <c r="Q6" s="7" t="n">
-        <v>21.623</v>
+        <v>22.633</v>
       </c>
     </row>
     <row r="7">
@@ -3802,25 +3802,25 @@
         <v>2</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>1.6</v>
+        <v>2</v>
       </c>
       <c r="H7" s="9" t="n">
-        <v>7.17</v>
+        <v>7.57</v>
       </c>
       <c r="I7" s="9" t="n">
-        <v>14.34</v>
+        <v>15.14</v>
       </c>
       <c r="J7" s="8" t="n"/>
       <c r="K7" s="8" t="n"/>
       <c r="L7" s="8" t="n"/>
       <c r="M7" s="8" t="n"/>
       <c r="N7" s="9" t="n">
-        <v>35.365</v>
+        <v>37.338</v>
       </c>
       <c r="O7" s="8" t="n"/>
       <c r="P7" s="8" t="n"/>
       <c r="Q7" s="9" t="n">
-        <v>35.365</v>
+        <v>37.338</v>
       </c>
     </row>
     <row r="8">
@@ -3843,25 +3843,25 @@
         <v>2</v>
       </c>
       <c r="G8" s="7" t="n">
-        <v>1.6</v>
+        <v>2</v>
       </c>
       <c r="H8" s="7" t="n">
-        <v>7.17</v>
+        <v>7.57</v>
       </c>
       <c r="I8" s="7" t="n">
-        <v>14.34</v>
+        <v>15.14</v>
       </c>
       <c r="J8" s="6" t="n"/>
       <c r="K8" s="6" t="n"/>
       <c r="L8" s="6" t="n"/>
       <c r="M8" s="6" t="n"/>
       <c r="N8" s="7" t="n">
-        <v>35.365</v>
+        <v>37.338</v>
       </c>
       <c r="O8" s="6" t="n"/>
       <c r="P8" s="6" t="n"/>
       <c r="Q8" s="7" t="n">
-        <v>35.365</v>
+        <v>37.338</v>
       </c>
     </row>
     <row r="9">
@@ -3886,16 +3886,16 @@
         <v>2</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>0.64</v>
+        <v>0.8</v>
       </c>
       <c r="H9" s="9" t="n">
-        <v>6.21</v>
+        <v>6.37</v>
       </c>
       <c r="I9" s="9" t="n">
-        <v>12.42</v>
+        <v>12.74</v>
       </c>
       <c r="J9" s="9" t="n">
-        <v>4.901</v>
+        <v>5.027</v>
       </c>
       <c r="K9" s="8" t="n"/>
       <c r="L9" s="8" t="n"/>
@@ -3904,7 +3904,7 @@
       <c r="O9" s="8" t="n"/>
       <c r="P9" s="8" t="n"/>
       <c r="Q9" s="9" t="n">
-        <v>4.901</v>
+        <v>5.027</v>
       </c>
     </row>
     <row r="10">
@@ -3970,25 +3970,25 @@
         <v>1</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>0.96</v>
+        <v>1.2</v>
       </c>
       <c r="H11" s="9" t="n">
-        <v>6.53</v>
+        <v>6.77</v>
       </c>
       <c r="I11" s="9" t="n">
-        <v>6.53</v>
+        <v>6.77</v>
       </c>
       <c r="J11" s="8" t="n"/>
       <c r="K11" s="8" t="n"/>
       <c r="L11" s="9" t="n">
-        <v>5.797</v>
+        <v>6.011</v>
       </c>
       <c r="M11" s="8" t="n"/>
       <c r="N11" s="8" t="n"/>
       <c r="O11" s="8" t="n"/>
       <c r="P11" s="8" t="n"/>
       <c r="Q11" s="9" t="n">
-        <v>5.797</v>
+        <v>6.011</v>
       </c>
     </row>
     <row r="12">
@@ -4011,25 +4011,25 @@
         <v>1</v>
       </c>
       <c r="G12" s="7" t="n">
-        <v>0.96</v>
+        <v>1.2</v>
       </c>
       <c r="H12" s="7" t="n">
-        <v>6.53</v>
+        <v>6.77</v>
       </c>
       <c r="I12" s="7" t="n">
-        <v>6.53</v>
+        <v>6.77</v>
       </c>
       <c r="J12" s="6" t="n"/>
       <c r="K12" s="6" t="n"/>
       <c r="L12" s="7" t="n">
-        <v>5.797</v>
+        <v>6.011</v>
       </c>
       <c r="M12" s="6" t="n"/>
       <c r="N12" s="6" t="n"/>
       <c r="O12" s="6" t="n"/>
       <c r="P12" s="6" t="n"/>
       <c r="Q12" s="7" t="n">
-        <v>5.797</v>
+        <v>6.011</v>
       </c>
     </row>
     <row r="13">
@@ -4052,25 +4052,25 @@
         <v>1</v>
       </c>
       <c r="G13" s="9" t="n">
-        <v>0.96</v>
+        <v>1.2</v>
       </c>
       <c r="H13" s="9" t="n">
-        <v>6.53</v>
+        <v>6.77</v>
       </c>
       <c r="I13" s="9" t="n">
-        <v>6.53</v>
+        <v>6.77</v>
       </c>
       <c r="J13" s="8" t="n"/>
       <c r="K13" s="8" t="n"/>
       <c r="L13" s="9" t="n">
-        <v>5.797</v>
+        <v>6.011</v>
       </c>
       <c r="M13" s="8" t="n"/>
       <c r="N13" s="8" t="n"/>
       <c r="O13" s="8" t="n"/>
       <c r="P13" s="8" t="n"/>
       <c r="Q13" s="9" t="n">
-        <v>5.797</v>
+        <v>6.011</v>
       </c>
     </row>
     <row r="14">
@@ -4109,7 +4109,7 @@
       <c r="O14" s="12" t="n"/>
       <c r="P14" s="12" t="n"/>
       <c r="Q14" s="12" t="n">
-        <v>109.1458905550298</v>
+        <v>114.1649995093697</v>
       </c>
     </row>
     <row r="15">
@@ -4132,25 +4132,25 @@
         <v>2</v>
       </c>
       <c r="G15" s="7" t="n">
-        <v>1.28</v>
+        <v>1.6</v>
       </c>
       <c r="H15" s="7" t="n">
-        <v>5.19</v>
+        <v>5.51</v>
       </c>
       <c r="I15" s="7" t="n">
-        <v>10.38</v>
+        <v>11.02</v>
       </c>
       <c r="J15" s="6" t="n"/>
       <c r="K15" s="6" t="n"/>
       <c r="L15" s="6" t="n"/>
       <c r="M15" s="7" t="n">
-        <v>16.383</v>
+        <v>17.393</v>
       </c>
       <c r="N15" s="6" t="n"/>
       <c r="O15" s="6" t="n"/>
       <c r="P15" s="6" t="n"/>
       <c r="Q15" s="7" t="n">
-        <v>16.383</v>
+        <v>17.393</v>
       </c>
     </row>
     <row r="16">
@@ -4173,25 +4173,25 @@
         <v>2</v>
       </c>
       <c r="G16" s="9" t="n">
-        <v>1.28</v>
+        <v>1.6</v>
       </c>
       <c r="H16" s="9" t="n">
-        <v>5.19</v>
+        <v>5.51</v>
       </c>
       <c r="I16" s="9" t="n">
-        <v>10.38</v>
+        <v>11.02</v>
       </c>
       <c r="J16" s="8" t="n"/>
       <c r="K16" s="8" t="n"/>
       <c r="L16" s="8" t="n"/>
       <c r="M16" s="9" t="n">
-        <v>16.383</v>
+        <v>17.393</v>
       </c>
       <c r="N16" s="8" t="n"/>
       <c r="O16" s="8" t="n"/>
       <c r="P16" s="8" t="n"/>
       <c r="Q16" s="9" t="n">
-        <v>16.383</v>
+        <v>17.393</v>
       </c>
     </row>
     <row r="17">
@@ -4214,25 +4214,25 @@
         <v>2</v>
       </c>
       <c r="G17" s="7" t="n">
-        <v>1.28</v>
+        <v>1.6</v>
       </c>
       <c r="H17" s="7" t="n">
-        <v>5.19</v>
+        <v>5.51</v>
       </c>
       <c r="I17" s="7" t="n">
-        <v>10.38</v>
+        <v>11.02</v>
       </c>
       <c r="J17" s="6" t="n"/>
       <c r="K17" s="6" t="n"/>
       <c r="L17" s="6" t="n"/>
       <c r="M17" s="7" t="n">
-        <v>16.383</v>
+        <v>17.393</v>
       </c>
       <c r="N17" s="6" t="n"/>
       <c r="O17" s="6" t="n"/>
       <c r="P17" s="6" t="n"/>
       <c r="Q17" s="7" t="n">
-        <v>16.383</v>
+        <v>17.393</v>
       </c>
     </row>
     <row r="18">
@@ -4255,25 +4255,25 @@
         <v>2</v>
       </c>
       <c r="G18" s="9" t="n">
-        <v>1.28</v>
+        <v>1.6</v>
       </c>
       <c r="H18" s="9" t="n">
-        <v>5.19</v>
+        <v>5.51</v>
       </c>
       <c r="I18" s="9" t="n">
-        <v>10.38</v>
+        <v>11.02</v>
       </c>
       <c r="J18" s="8" t="n"/>
       <c r="K18" s="8" t="n"/>
       <c r="L18" s="8" t="n"/>
       <c r="M18" s="9" t="n">
-        <v>16.383</v>
+        <v>17.393</v>
       </c>
       <c r="N18" s="8" t="n"/>
       <c r="O18" s="8" t="n"/>
       <c r="P18" s="8" t="n"/>
       <c r="Q18" s="9" t="n">
-        <v>16.383</v>
+        <v>17.393</v>
       </c>
     </row>
     <row r="19">
@@ -4298,16 +4298,16 @@
         <v>2</v>
       </c>
       <c r="G19" s="7" t="n">
-        <v>0.64</v>
+        <v>0.8</v>
       </c>
       <c r="H19" s="7" t="n">
-        <v>4.55</v>
+        <v>4.71</v>
       </c>
       <c r="I19" s="7" t="n">
-        <v>9.1</v>
+        <v>9.42</v>
       </c>
       <c r="J19" s="7" t="n">
-        <v>3.591</v>
+        <v>3.717</v>
       </c>
       <c r="K19" s="6" t="n"/>
       <c r="L19" s="6" t="n"/>
@@ -4316,7 +4316,7 @@
       <c r="O19" s="6" t="n"/>
       <c r="P19" s="6" t="n"/>
       <c r="Q19" s="7" t="n">
-        <v>3.591</v>
+        <v>3.717</v>
       </c>
     </row>
     <row r="20">
@@ -4382,25 +4382,25 @@
         <v>1</v>
       </c>
       <c r="G21" s="7" t="n">
-        <v>0.96</v>
+        <v>1.2</v>
       </c>
       <c r="H21" s="7" t="n">
-        <v>4.87</v>
+        <v>5.11</v>
       </c>
       <c r="I21" s="7" t="n">
-        <v>4.87</v>
+        <v>5.11</v>
       </c>
       <c r="J21" s="6" t="n"/>
       <c r="K21" s="6" t="n"/>
       <c r="L21" s="7" t="n">
-        <v>4.324</v>
+        <v>4.537</v>
       </c>
       <c r="M21" s="6" t="n"/>
       <c r="N21" s="6" t="n"/>
       <c r="O21" s="6" t="n"/>
       <c r="P21" s="6" t="n"/>
       <c r="Q21" s="7" t="n">
-        <v>4.324</v>
+        <v>4.537</v>
       </c>
     </row>
     <row r="22">
@@ -4423,25 +4423,25 @@
         <v>1</v>
       </c>
       <c r="G22" s="9" t="n">
-        <v>0.96</v>
+        <v>1.2</v>
       </c>
       <c r="H22" s="9" t="n">
-        <v>4.87</v>
+        <v>5.11</v>
       </c>
       <c r="I22" s="9" t="n">
-        <v>4.87</v>
+        <v>5.11</v>
       </c>
       <c r="J22" s="8" t="n"/>
       <c r="K22" s="8" t="n"/>
       <c r="L22" s="9" t="n">
-        <v>4.324</v>
+        <v>4.537</v>
       </c>
       <c r="M22" s="8" t="n"/>
       <c r="N22" s="8" t="n"/>
       <c r="O22" s="8" t="n"/>
       <c r="P22" s="8" t="n"/>
       <c r="Q22" s="9" t="n">
-        <v>4.324</v>
+        <v>4.537</v>
       </c>
     </row>
     <row r="23">
@@ -4464,25 +4464,25 @@
         <v>1</v>
       </c>
       <c r="G23" s="7" t="n">
-        <v>0.96</v>
+        <v>1.2</v>
       </c>
       <c r="H23" s="7" t="n">
-        <v>4.87</v>
+        <v>5.11</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>4.87</v>
+        <v>5.11</v>
       </c>
       <c r="J23" s="6" t="n"/>
       <c r="K23" s="6" t="n"/>
       <c r="L23" s="7" t="n">
-        <v>4.324</v>
+        <v>4.537</v>
       </c>
       <c r="M23" s="6" t="n"/>
       <c r="N23" s="6" t="n"/>
       <c r="O23" s="6" t="n"/>
       <c r="P23" s="6" t="n"/>
       <c r="Q23" s="7" t="n">
-        <v>4.324</v>
+        <v>4.537</v>
       </c>
     </row>
     <row r="24">
@@ -4505,25 +4505,25 @@
         <v>1</v>
       </c>
       <c r="G24" s="9" t="n">
-        <v>0.96</v>
+        <v>1.2</v>
       </c>
       <c r="H24" s="9" t="n">
-        <v>4.87</v>
+        <v>5.11</v>
       </c>
       <c r="I24" s="9" t="n">
-        <v>4.87</v>
+        <v>5.11</v>
       </c>
       <c r="J24" s="8" t="n"/>
       <c r="K24" s="8" t="n"/>
       <c r="L24" s="9" t="n">
-        <v>4.324</v>
+        <v>4.537</v>
       </c>
       <c r="M24" s="8" t="n"/>
       <c r="N24" s="8" t="n"/>
       <c r="O24" s="8" t="n"/>
       <c r="P24" s="8" t="n"/>
       <c r="Q24" s="9" t="n">
-        <v>4.324</v>
+        <v>4.537</v>
       </c>
     </row>
     <row r="25">
@@ -4912,7 +4912,7 @@
       <c r="O35" s="12" t="n"/>
       <c r="P35" s="12" t="n"/>
       <c r="Q35" s="12" t="n">
-        <v>109.8159435733543</v>
+        <v>115.577980285406</v>
       </c>
     </row>
     <row r="36">
@@ -4935,25 +4935,25 @@
         <v>2</v>
       </c>
       <c r="G36" s="7" t="n">
-        <v>1.28</v>
+        <v>1.6</v>
       </c>
       <c r="H36" s="7" t="n">
-        <v>5.56</v>
+        <v>5.88</v>
       </c>
       <c r="I36" s="7" t="n">
-        <v>11.12</v>
+        <v>11.76</v>
       </c>
       <c r="J36" s="6" t="n"/>
       <c r="K36" s="6" t="n"/>
       <c r="L36" s="6" t="n"/>
       <c r="M36" s="7" t="n">
-        <v>17.551</v>
+        <v>18.561</v>
       </c>
       <c r="N36" s="6" t="n"/>
       <c r="O36" s="6" t="n"/>
       <c r="P36" s="6" t="n"/>
       <c r="Q36" s="7" t="n">
-        <v>17.551</v>
+        <v>18.561</v>
       </c>
     </row>
     <row r="37">
@@ -4976,25 +4976,25 @@
         <v>2</v>
       </c>
       <c r="G37" s="9" t="n">
-        <v>0.96</v>
+        <v>1.2</v>
       </c>
       <c r="H37" s="9" t="n">
-        <v>5.24</v>
+        <v>5.48</v>
       </c>
       <c r="I37" s="9" t="n">
-        <v>10.48</v>
+        <v>10.96</v>
       </c>
       <c r="J37" s="8" t="n"/>
       <c r="K37" s="8" t="n"/>
       <c r="L37" s="9" t="n">
-        <v>9.304</v>
+        <v>9.73</v>
       </c>
       <c r="M37" s="8" t="n"/>
       <c r="N37" s="8" t="n"/>
       <c r="O37" s="8" t="n"/>
       <c r="P37" s="8" t="n"/>
       <c r="Q37" s="9" t="n">
-        <v>9.304</v>
+        <v>9.73</v>
       </c>
     </row>
     <row r="38">
@@ -5017,25 +5017,25 @@
         <v>2</v>
       </c>
       <c r="G38" s="7" t="n">
-        <v>1.6</v>
+        <v>2</v>
       </c>
       <c r="H38" s="7" t="n">
-        <v>5.88</v>
+        <v>6.28</v>
       </c>
       <c r="I38" s="7" t="n">
-        <v>11.76</v>
+        <v>12.56</v>
       </c>
       <c r="J38" s="6" t="n"/>
       <c r="K38" s="6" t="n"/>
       <c r="L38" s="6" t="n"/>
       <c r="M38" s="6" t="n"/>
       <c r="N38" s="7" t="n">
-        <v>29.002</v>
+        <v>30.975</v>
       </c>
       <c r="O38" s="6" t="n"/>
       <c r="P38" s="6" t="n"/>
       <c r="Q38" s="7" t="n">
-        <v>29.002</v>
+        <v>30.975</v>
       </c>
     </row>
     <row r="39">
@@ -5230,13 +5230,13 @@
         <v>1</v>
       </c>
       <c r="G43" s="9" t="n">
-        <v>2</v>
+        <v>2.5</v>
       </c>
       <c r="H43" s="9" t="n">
-        <v>6.28</v>
+        <v>6.78</v>
       </c>
       <c r="I43" s="9" t="n">
-        <v>6.28</v>
+        <v>6.78</v>
       </c>
       <c r="J43" s="8" t="n"/>
       <c r="K43" s="8" t="n"/>
@@ -5244,11 +5244,11 @@
       <c r="M43" s="8" t="n"/>
       <c r="N43" s="8" t="n"/>
       <c r="O43" s="9" t="n">
-        <v>24.199</v>
+        <v>26.126</v>
       </c>
       <c r="P43" s="8" t="n"/>
       <c r="Q43" s="9" t="n">
-        <v>24.199</v>
+        <v>26.126</v>
       </c>
     </row>
     <row r="44">
@@ -5271,25 +5271,25 @@
         <v>1</v>
       </c>
       <c r="G44" s="7" t="n">
-        <v>0.96</v>
+        <v>1.2</v>
       </c>
       <c r="H44" s="7" t="n">
-        <v>5.24</v>
+        <v>5.48</v>
       </c>
       <c r="I44" s="7" t="n">
-        <v>5.24</v>
+        <v>5.48</v>
       </c>
       <c r="J44" s="6" t="n"/>
       <c r="K44" s="6" t="n"/>
       <c r="L44" s="7" t="n">
-        <v>4.652</v>
+        <v>4.865</v>
       </c>
       <c r="M44" s="6" t="n"/>
       <c r="N44" s="6" t="n"/>
       <c r="O44" s="6" t="n"/>
       <c r="P44" s="6" t="n"/>
       <c r="Q44" s="7" t="n">
-        <v>4.652</v>
+        <v>4.865</v>
       </c>
     </row>
     <row r="45">
@@ -5312,25 +5312,25 @@
         <v>1</v>
       </c>
       <c r="G45" s="9" t="n">
-        <v>0.96</v>
+        <v>1.2</v>
       </c>
       <c r="H45" s="9" t="n">
-        <v>5.24</v>
+        <v>5.48</v>
       </c>
       <c r="I45" s="9" t="n">
-        <v>5.24</v>
+        <v>5.48</v>
       </c>
       <c r="J45" s="8" t="n"/>
       <c r="K45" s="8" t="n"/>
       <c r="L45" s="9" t="n">
-        <v>4.652</v>
+        <v>4.865</v>
       </c>
       <c r="M45" s="8" t="n"/>
       <c r="N45" s="8" t="n"/>
       <c r="O45" s="8" t="n"/>
       <c r="P45" s="8" t="n"/>
       <c r="Q45" s="9" t="n">
-        <v>4.652</v>
+        <v>4.865</v>
       </c>
     </row>
     <row r="46">
@@ -7084,7 +7084,7 @@
       <c r="O95" s="12" t="n"/>
       <c r="P95" s="12" t="n"/>
       <c r="Q95" s="12" t="n">
-        <v>71.15139360429113</v>
+        <v>76.17050255863109</v>
       </c>
     </row>
     <row r="96">
@@ -7107,25 +7107,25 @@
         <v>2</v>
       </c>
       <c r="G96" s="7" t="n">
-        <v>1.28</v>
+        <v>1.6</v>
       </c>
       <c r="H96" s="7" t="n">
-        <v>3.52</v>
+        <v>3.84</v>
       </c>
       <c r="I96" s="7" t="n">
-        <v>7.04</v>
+        <v>7.68</v>
       </c>
       <c r="J96" s="6" t="n"/>
       <c r="K96" s="6" t="n"/>
       <c r="L96" s="6" t="n"/>
       <c r="M96" s="7" t="n">
-        <v>11.111</v>
+        <v>12.122</v>
       </c>
       <c r="N96" s="6" t="n"/>
       <c r="O96" s="6" t="n"/>
       <c r="P96" s="6" t="n"/>
       <c r="Q96" s="7" t="n">
-        <v>11.111</v>
+        <v>12.122</v>
       </c>
     </row>
     <row r="97">
@@ -7148,25 +7148,25 @@
         <v>2</v>
       </c>
       <c r="G97" s="9" t="n">
-        <v>1.28</v>
+        <v>1.6</v>
       </c>
       <c r="H97" s="9" t="n">
-        <v>3.52</v>
+        <v>3.84</v>
       </c>
       <c r="I97" s="9" t="n">
-        <v>7.04</v>
+        <v>7.68</v>
       </c>
       <c r="J97" s="8" t="n"/>
       <c r="K97" s="8" t="n"/>
       <c r="L97" s="8" t="n"/>
       <c r="M97" s="9" t="n">
-        <v>11.111</v>
+        <v>12.122</v>
       </c>
       <c r="N97" s="8" t="n"/>
       <c r="O97" s="8" t="n"/>
       <c r="P97" s="8" t="n"/>
       <c r="Q97" s="9" t="n">
-        <v>11.111</v>
+        <v>12.122</v>
       </c>
     </row>
     <row r="98">
@@ -7189,25 +7189,25 @@
         <v>2</v>
       </c>
       <c r="G98" s="7" t="n">
-        <v>1.28</v>
+        <v>1.6</v>
       </c>
       <c r="H98" s="7" t="n">
-        <v>3.52</v>
+        <v>3.84</v>
       </c>
       <c r="I98" s="7" t="n">
-        <v>7.04</v>
+        <v>7.68</v>
       </c>
       <c r="J98" s="6" t="n"/>
       <c r="K98" s="6" t="n"/>
       <c r="L98" s="6" t="n"/>
       <c r="M98" s="7" t="n">
-        <v>11.111</v>
+        <v>12.122</v>
       </c>
       <c r="N98" s="6" t="n"/>
       <c r="O98" s="6" t="n"/>
       <c r="P98" s="6" t="n"/>
       <c r="Q98" s="7" t="n">
-        <v>11.111</v>
+        <v>12.122</v>
       </c>
     </row>
     <row r="99">
@@ -7230,25 +7230,25 @@
         <v>2</v>
       </c>
       <c r="G99" s="9" t="n">
-        <v>1.28</v>
+        <v>1.6</v>
       </c>
       <c r="H99" s="9" t="n">
-        <v>3.52</v>
+        <v>3.84</v>
       </c>
       <c r="I99" s="9" t="n">
-        <v>7.04</v>
+        <v>7.68</v>
       </c>
       <c r="J99" s="8" t="n"/>
       <c r="K99" s="8" t="n"/>
       <c r="L99" s="8" t="n"/>
       <c r="M99" s="9" t="n">
-        <v>11.111</v>
+        <v>12.122</v>
       </c>
       <c r="N99" s="8" t="n"/>
       <c r="O99" s="8" t="n"/>
       <c r="P99" s="8" t="n"/>
       <c r="Q99" s="9" t="n">
-        <v>11.111</v>
+        <v>12.122</v>
       </c>
     </row>
     <row r="100">
@@ -7273,16 +7273,16 @@
         <v>2</v>
       </c>
       <c r="G100" s="7" t="n">
-        <v>0.64</v>
+        <v>0.8</v>
       </c>
       <c r="H100" s="7" t="n">
-        <v>2.88</v>
+        <v>3.04</v>
       </c>
       <c r="I100" s="7" t="n">
-        <v>5.76</v>
+        <v>6.08</v>
       </c>
       <c r="J100" s="7" t="n">
-        <v>2.273</v>
+        <v>2.399</v>
       </c>
       <c r="K100" s="6" t="n"/>
       <c r="L100" s="6" t="n"/>
@@ -7291,7 +7291,7 @@
       <c r="O100" s="6" t="n"/>
       <c r="P100" s="6" t="n"/>
       <c r="Q100" s="7" t="n">
-        <v>2.273</v>
+        <v>2.399</v>
       </c>
     </row>
     <row r="101">
@@ -7357,25 +7357,25 @@
         <v>1</v>
       </c>
       <c r="G102" s="7" t="n">
-        <v>0.96</v>
+        <v>1.2</v>
       </c>
       <c r="H102" s="7" t="n">
-        <v>3.2</v>
+        <v>3.44</v>
       </c>
       <c r="I102" s="7" t="n">
-        <v>3.2</v>
+        <v>3.44</v>
       </c>
       <c r="J102" s="6" t="n"/>
       <c r="K102" s="6" t="n"/>
       <c r="L102" s="7" t="n">
-        <v>2.841</v>
+        <v>3.054</v>
       </c>
       <c r="M102" s="6" t="n"/>
       <c r="N102" s="6" t="n"/>
       <c r="O102" s="6" t="n"/>
       <c r="P102" s="6" t="n"/>
       <c r="Q102" s="7" t="n">
-        <v>2.841</v>
+        <v>3.054</v>
       </c>
     </row>
     <row r="103">
@@ -7398,25 +7398,25 @@
         <v>1</v>
       </c>
       <c r="G103" s="9" t="n">
-        <v>0.96</v>
+        <v>1.2</v>
       </c>
       <c r="H103" s="9" t="n">
-        <v>3.2</v>
+        <v>3.44</v>
       </c>
       <c r="I103" s="9" t="n">
-        <v>3.2</v>
+        <v>3.44</v>
       </c>
       <c r="J103" s="8" t="n"/>
       <c r="K103" s="8" t="n"/>
       <c r="L103" s="9" t="n">
-        <v>2.841</v>
+        <v>3.054</v>
       </c>
       <c r="M103" s="8" t="n"/>
       <c r="N103" s="8" t="n"/>
       <c r="O103" s="8" t="n"/>
       <c r="P103" s="8" t="n"/>
       <c r="Q103" s="9" t="n">
-        <v>2.841</v>
+        <v>3.054</v>
       </c>
     </row>
     <row r="104">
@@ -7439,25 +7439,25 @@
         <v>1</v>
       </c>
       <c r="G104" s="7" t="n">
-        <v>0.96</v>
+        <v>1.2</v>
       </c>
       <c r="H104" s="7" t="n">
-        <v>3.2</v>
+        <v>3.44</v>
       </c>
       <c r="I104" s="7" t="n">
-        <v>3.2</v>
+        <v>3.44</v>
       </c>
       <c r="J104" s="6" t="n"/>
       <c r="K104" s="6" t="n"/>
       <c r="L104" s="7" t="n">
-        <v>2.841</v>
+        <v>3.054</v>
       </c>
       <c r="M104" s="6" t="n"/>
       <c r="N104" s="6" t="n"/>
       <c r="O104" s="6" t="n"/>
       <c r="P104" s="6" t="n"/>
       <c r="Q104" s="7" t="n">
-        <v>2.841</v>
+        <v>3.054</v>
       </c>
     </row>
     <row r="105">
@@ -7480,25 +7480,25 @@
         <v>1</v>
       </c>
       <c r="G105" s="9" t="n">
-        <v>0.96</v>
+        <v>1.2</v>
       </c>
       <c r="H105" s="9" t="n">
-        <v>3.2</v>
+        <v>3.44</v>
       </c>
       <c r="I105" s="9" t="n">
-        <v>3.2</v>
+        <v>3.44</v>
       </c>
       <c r="J105" s="8" t="n"/>
       <c r="K105" s="8" t="n"/>
       <c r="L105" s="9" t="n">
-        <v>2.841</v>
+        <v>3.054</v>
       </c>
       <c r="M105" s="8" t="n"/>
       <c r="N105" s="8" t="n"/>
       <c r="O105" s="8" t="n"/>
       <c r="P105" s="8" t="n"/>
       <c r="Q105" s="9" t="n">
-        <v>2.841</v>
+        <v>3.054</v>
       </c>
     </row>
     <row r="106">
@@ -7537,7 +7537,7 @@
       <c r="O106" s="12" t="n"/>
       <c r="P106" s="12" t="n"/>
       <c r="Q106" s="12" t="n">
-        <v>88.93135032461809</v>
+        <v>93.95045927895805</v>
       </c>
     </row>
     <row r="107">
@@ -7560,25 +7560,25 @@
         <v>2</v>
       </c>
       <c r="G107" s="7" t="n">
-        <v>1.28</v>
+        <v>1.6</v>
       </c>
       <c r="H107" s="7" t="n">
-        <v>4.3</v>
+        <v>4.62</v>
       </c>
       <c r="I107" s="7" t="n">
-        <v>8.6</v>
+        <v>9.24</v>
       </c>
       <c r="J107" s="6" t="n"/>
       <c r="K107" s="6" t="n"/>
       <c r="L107" s="6" t="n"/>
       <c r="M107" s="7" t="n">
-        <v>13.574</v>
+        <v>14.584</v>
       </c>
       <c r="N107" s="6" t="n"/>
       <c r="O107" s="6" t="n"/>
       <c r="P107" s="6" t="n"/>
       <c r="Q107" s="7" t="n">
-        <v>13.574</v>
+        <v>14.584</v>
       </c>
     </row>
     <row r="108">
@@ -7601,25 +7601,25 @@
         <v>2</v>
       </c>
       <c r="G108" s="9" t="n">
-        <v>1.28</v>
+        <v>1.6</v>
       </c>
       <c r="H108" s="9" t="n">
-        <v>4.3</v>
+        <v>4.62</v>
       </c>
       <c r="I108" s="9" t="n">
-        <v>8.6</v>
+        <v>9.24</v>
       </c>
       <c r="J108" s="8" t="n"/>
       <c r="K108" s="8" t="n"/>
       <c r="L108" s="8" t="n"/>
       <c r="M108" s="9" t="n">
-        <v>13.574</v>
+        <v>14.584</v>
       </c>
       <c r="N108" s="8" t="n"/>
       <c r="O108" s="8" t="n"/>
       <c r="P108" s="8" t="n"/>
       <c r="Q108" s="9" t="n">
-        <v>13.574</v>
+        <v>14.584</v>
       </c>
     </row>
     <row r="109">
@@ -7642,25 +7642,25 @@
         <v>2</v>
       </c>
       <c r="G109" s="7" t="n">
-        <v>1.28</v>
+        <v>1.6</v>
       </c>
       <c r="H109" s="7" t="n">
-        <v>4.3</v>
+        <v>4.62</v>
       </c>
       <c r="I109" s="7" t="n">
-        <v>8.6</v>
+        <v>9.24</v>
       </c>
       <c r="J109" s="6" t="n"/>
       <c r="K109" s="6" t="n"/>
       <c r="L109" s="6" t="n"/>
       <c r="M109" s="7" t="n">
-        <v>13.574</v>
+        <v>14.584</v>
       </c>
       <c r="N109" s="6" t="n"/>
       <c r="O109" s="6" t="n"/>
       <c r="P109" s="6" t="n"/>
       <c r="Q109" s="7" t="n">
-        <v>13.574</v>
+        <v>14.584</v>
       </c>
     </row>
     <row r="110">
@@ -7683,25 +7683,25 @@
         <v>2</v>
       </c>
       <c r="G110" s="9" t="n">
-        <v>1.28</v>
+        <v>1.6</v>
       </c>
       <c r="H110" s="9" t="n">
-        <v>4.3</v>
+        <v>4.62</v>
       </c>
       <c r="I110" s="9" t="n">
-        <v>8.6</v>
+        <v>9.24</v>
       </c>
       <c r="J110" s="8" t="n"/>
       <c r="K110" s="8" t="n"/>
       <c r="L110" s="8" t="n"/>
       <c r="M110" s="9" t="n">
-        <v>13.574</v>
+        <v>14.584</v>
       </c>
       <c r="N110" s="8" t="n"/>
       <c r="O110" s="8" t="n"/>
       <c r="P110" s="8" t="n"/>
       <c r="Q110" s="9" t="n">
-        <v>13.574</v>
+        <v>14.584</v>
       </c>
     </row>
     <row r="111">
@@ -7726,16 +7726,16 @@
         <v>2</v>
       </c>
       <c r="G111" s="7" t="n">
-        <v>0.64</v>
+        <v>0.8</v>
       </c>
       <c r="H111" s="7" t="n">
-        <v>3.66</v>
+        <v>3.82</v>
       </c>
       <c r="I111" s="7" t="n">
-        <v>7.32</v>
+        <v>7.64</v>
       </c>
       <c r="J111" s="7" t="n">
-        <v>2.888</v>
+        <v>3.015</v>
       </c>
       <c r="K111" s="6" t="n"/>
       <c r="L111" s="6" t="n"/>
@@ -7744,7 +7744,7 @@
       <c r="O111" s="6" t="n"/>
       <c r="P111" s="6" t="n"/>
       <c r="Q111" s="7" t="n">
-        <v>2.888</v>
+        <v>3.015</v>
       </c>
     </row>
     <row r="112">
@@ -7810,25 +7810,25 @@
         <v>1</v>
       </c>
       <c r="G113" s="7" t="n">
-        <v>0.96</v>
+        <v>1.2</v>
       </c>
       <c r="H113" s="7" t="n">
-        <v>3.98</v>
+        <v>4.22</v>
       </c>
       <c r="I113" s="7" t="n">
-        <v>3.98</v>
+        <v>4.22</v>
       </c>
       <c r="J113" s="6" t="n"/>
       <c r="K113" s="6" t="n"/>
       <c r="L113" s="7" t="n">
-        <v>3.534</v>
+        <v>3.747</v>
       </c>
       <c r="M113" s="6" t="n"/>
       <c r="N113" s="6" t="n"/>
       <c r="O113" s="6" t="n"/>
       <c r="P113" s="6" t="n"/>
       <c r="Q113" s="7" t="n">
-        <v>3.534</v>
+        <v>3.747</v>
       </c>
     </row>
     <row r="114">
@@ -7851,25 +7851,25 @@
         <v>1</v>
       </c>
       <c r="G114" s="9" t="n">
-        <v>0.96</v>
+        <v>1.2</v>
       </c>
       <c r="H114" s="9" t="n">
-        <v>3.98</v>
+        <v>4.22</v>
       </c>
       <c r="I114" s="9" t="n">
-        <v>3.98</v>
+        <v>4.22</v>
       </c>
       <c r="J114" s="8" t="n"/>
       <c r="K114" s="8" t="n"/>
       <c r="L114" s="9" t="n">
-        <v>3.534</v>
+        <v>3.747</v>
       </c>
       <c r="M114" s="8" t="n"/>
       <c r="N114" s="8" t="n"/>
       <c r="O114" s="8" t="n"/>
       <c r="P114" s="8" t="n"/>
       <c r="Q114" s="9" t="n">
-        <v>3.534</v>
+        <v>3.747</v>
       </c>
     </row>
     <row r="115">
@@ -7892,25 +7892,25 @@
         <v>1</v>
       </c>
       <c r="G115" s="7" t="n">
-        <v>0.96</v>
+        <v>1.2</v>
       </c>
       <c r="H115" s="7" t="n">
-        <v>3.98</v>
+        <v>4.22</v>
       </c>
       <c r="I115" s="7" t="n">
-        <v>3.98</v>
+        <v>4.22</v>
       </c>
       <c r="J115" s="6" t="n"/>
       <c r="K115" s="6" t="n"/>
       <c r="L115" s="7" t="n">
-        <v>3.534</v>
+        <v>3.747</v>
       </c>
       <c r="M115" s="6" t="n"/>
       <c r="N115" s="6" t="n"/>
       <c r="O115" s="6" t="n"/>
       <c r="P115" s="6" t="n"/>
       <c r="Q115" s="7" t="n">
-        <v>3.534</v>
+        <v>3.747</v>
       </c>
     </row>
     <row r="116">
@@ -7933,25 +7933,25 @@
         <v>1</v>
       </c>
       <c r="G116" s="9" t="n">
-        <v>0.96</v>
+        <v>1.2</v>
       </c>
       <c r="H116" s="9" t="n">
-        <v>3.98</v>
+        <v>4.22</v>
       </c>
       <c r="I116" s="9" t="n">
-        <v>3.98</v>
+        <v>4.22</v>
       </c>
       <c r="J116" s="8" t="n"/>
       <c r="K116" s="8" t="n"/>
       <c r="L116" s="9" t="n">
-        <v>3.534</v>
+        <v>3.747</v>
       </c>
       <c r="M116" s="8" t="n"/>
       <c r="N116" s="8" t="n"/>
       <c r="O116" s="8" t="n"/>
       <c r="P116" s="8" t="n"/>
       <c r="Q116" s="9" t="n">
-        <v>3.534</v>
+        <v>3.747</v>
       </c>
     </row>
     <row r="117">
@@ -8015,7 +8015,7 @@
         </is>
       </c>
       <c r="B120" s="16" t="n">
-        <v>107.974</v>
+        <v>108.479</v>
       </c>
     </row>
     <row r="121">
@@ -8035,7 +8035,7 @@
         </is>
       </c>
       <c r="B122" s="16" t="n">
-        <v>78.795</v>
+        <v>82.845</v>
       </c>
     </row>
     <row r="123">
@@ -8045,7 +8045,7 @@
         </is>
       </c>
       <c r="B123" s="16" t="n">
-        <v>246.692</v>
+        <v>262.856</v>
       </c>
     </row>
     <row r="124">
@@ -8055,7 +8055,7 @@
         </is>
       </c>
       <c r="B124" s="16" t="n">
-        <v>99.732</v>
+        <v>105.651</v>
       </c>
     </row>
     <row r="125">
@@ -8065,7 +8065,7 @@
         </is>
       </c>
       <c r="B125" s="16" t="n">
-        <v>24.199</v>
+        <v>26.126</v>
       </c>
     </row>
     <row r="126">
@@ -8085,7 +8085,7 @@
         </is>
       </c>
       <c r="B127" s="18" t="n">
-        <v>608.491</v>
+        <v>637.056</v>
       </c>
     </row>
   </sheetData>
@@ -8177,19 +8177,19 @@
         </is>
       </c>
       <c r="B3" s="7" t="n">
-        <v>4.901</v>
+        <v>5.027</v>
       </c>
       <c r="C3" s="7" t="n">
-        <v>51.099</v>
+        <v>50.408</v>
       </c>
       <c r="D3" s="7" t="n">
-        <v>17.392</v>
+        <v>18.032</v>
       </c>
       <c r="E3" s="7" t="n">
-        <v>64.87</v>
+        <v>67.90000000000001</v>
       </c>
       <c r="F3" s="7" t="n">
-        <v>70.729</v>
+        <v>74.675</v>
       </c>
       <c r="G3" s="7" t="n">
         <v>0</v>
@@ -8198,7 +8198,7 @@
         <v>0</v>
       </c>
       <c r="I3" s="7" t="n">
-        <v>208.99</v>
+        <v>216.042</v>
       </c>
     </row>
     <row r="4">
@@ -8208,16 +8208,16 @@
         </is>
       </c>
       <c r="B4" s="9" t="n">
-        <v>26.319</v>
+        <v>26.445</v>
       </c>
       <c r="C4" s="9" t="n">
         <v>0</v>
       </c>
       <c r="D4" s="9" t="n">
-        <v>17.295</v>
+        <v>18.147</v>
       </c>
       <c r="E4" s="9" t="n">
-        <v>65.533</v>
+        <v>69.57299999999999</v>
       </c>
       <c r="F4" s="9" t="n">
         <v>0</v>
@@ -8229,7 +8229,7 @@
         <v>0</v>
       </c>
       <c r="I4" s="9" t="n">
-        <v>109.146</v>
+        <v>114.165</v>
       </c>
     </row>
     <row r="5">
@@ -8555,22 +8555,22 @@
         <v>0</v>
       </c>
       <c r="D15" s="7" t="n">
-        <v>18.609</v>
+        <v>19.461</v>
       </c>
       <c r="E15" s="7" t="n">
-        <v>17.551</v>
+        <v>18.561</v>
       </c>
       <c r="F15" s="7" t="n">
-        <v>29.002</v>
+        <v>30.975</v>
       </c>
       <c r="G15" s="7" t="n">
-        <v>24.199</v>
+        <v>26.126</v>
       </c>
       <c r="H15" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I15" s="7" t="n">
-        <v>109.816</v>
+        <v>115.578</v>
       </c>
     </row>
     <row r="16">
@@ -10099,16 +10099,16 @@
         </is>
       </c>
       <c r="B65" s="7" t="n">
-        <v>15.341</v>
+        <v>15.468</v>
       </c>
       <c r="C65" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D65" s="7" t="n">
-        <v>11.364</v>
+        <v>12.216</v>
       </c>
       <c r="E65" s="7" t="n">
-        <v>44.446</v>
+        <v>48.486</v>
       </c>
       <c r="F65" s="7" t="n">
         <v>0</v>
@@ -10120,7 +10120,7 @@
         <v>0</v>
       </c>
       <c r="I65" s="7" t="n">
-        <v>71.151</v>
+        <v>76.17100000000001</v>
       </c>
     </row>
     <row r="66">
@@ -10130,16 +10130,16 @@
         </is>
       </c>
       <c r="B66" s="9" t="n">
-        <v>20.503</v>
+        <v>20.629</v>
       </c>
       <c r="C66" s="9" t="n">
         <v>0</v>
       </c>
       <c r="D66" s="9" t="n">
-        <v>14.134</v>
+        <v>14.986</v>
       </c>
       <c r="E66" s="9" t="n">
-        <v>54.295</v>
+        <v>58.335</v>
       </c>
       <c r="F66" s="9" t="n">
         <v>0</v>
@@ -10151,7 +10151,7 @@
         <v>0</v>
       </c>
       <c r="I66" s="9" t="n">
-        <v>88.931</v>
+        <v>93.95</v>
       </c>
     </row>
     <row r="67">
@@ -10192,28 +10192,28 @@
         </is>
       </c>
       <c r="B68" s="11" t="n">
-        <v>87.51900000000001</v>
+        <v>88.024</v>
       </c>
       <c r="C68" s="11" t="n">
-        <v>51.099</v>
+        <v>50.408</v>
       </c>
       <c r="D68" s="11" t="n">
-        <v>78.79300000000001</v>
+        <v>82.842</v>
       </c>
       <c r="E68" s="11" t="n">
-        <v>246.694</v>
+        <v>262.856</v>
       </c>
       <c r="F68" s="11" t="n">
-        <v>99.73099999999999</v>
+        <v>105.65</v>
       </c>
       <c r="G68" s="11" t="n">
-        <v>24.199</v>
+        <v>26.126</v>
       </c>
       <c r="H68" s="11" t="n">
         <v>0</v>
       </c>
       <c r="I68" s="11" t="n">
-        <v>588.035</v>
+        <v>615.9059999999999</v>
       </c>
     </row>
   </sheetData>
@@ -10284,13 +10284,13 @@
         <v>9</v>
       </c>
       <c r="C3" s="7" t="n">
-        <v>221800</v>
+        <v>223080</v>
       </c>
       <c r="D3" s="7" t="n">
-        <v>87.51900000000001</v>
+        <v>88.024</v>
       </c>
       <c r="E3" s="7" t="n">
-        <v>14.88</v>
+        <v>14.29</v>
       </c>
     </row>
     <row r="4">
@@ -10303,13 +10303,13 @@
         <v>1</v>
       </c>
       <c r="C4" s="9" t="n">
-        <v>82880</v>
+        <v>81760</v>
       </c>
       <c r="D4" s="9" t="n">
-        <v>51.099</v>
+        <v>50.408</v>
       </c>
       <c r="E4" s="9" t="n">
-        <v>8.69</v>
+        <v>8.18</v>
       </c>
     </row>
     <row r="5">
@@ -10322,13 +10322,13 @@
         <v>18</v>
       </c>
       <c r="C5" s="7" t="n">
-        <v>88750</v>
+        <v>93310</v>
       </c>
       <c r="D5" s="7" t="n">
-        <v>78.79300000000001</v>
+        <v>82.842</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>13.4</v>
+        <v>13.45</v>
       </c>
     </row>
     <row r="6">
@@ -10341,13 +10341,13 @@
         <v>16</v>
       </c>
       <c r="C6" s="9" t="n">
-        <v>156300</v>
+        <v>166540</v>
       </c>
       <c r="D6" s="9" t="n">
-        <v>246.694</v>
+        <v>262.856</v>
       </c>
       <c r="E6" s="9" t="n">
-        <v>41.95</v>
+        <v>42.68</v>
       </c>
     </row>
     <row r="7">
@@ -10360,13 +10360,13 @@
         <v>3</v>
       </c>
       <c r="C7" s="7" t="n">
-        <v>40440</v>
+        <v>42840</v>
       </c>
       <c r="D7" s="7" t="n">
-        <v>99.73099999999999</v>
+        <v>105.65</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>16.96</v>
+        <v>17.15</v>
       </c>
     </row>
     <row r="8">
@@ -10379,13 +10379,13 @@
         <v>1</v>
       </c>
       <c r="C8" s="9" t="n">
-        <v>6280</v>
+        <v>6780</v>
       </c>
       <c r="D8" s="9" t="n">
-        <v>24.199</v>
+        <v>26.126</v>
       </c>
       <c r="E8" s="9" t="n">
-        <v>4.12</v>
+        <v>4.24</v>
       </c>
     </row>
     <row r="9">
@@ -10399,7 +10399,7 @@
       </c>
       <c r="C9" s="10" t="n"/>
       <c r="D9" s="11" t="n">
-        <v>588.035</v>
+        <v>615.9059999999999</v>
       </c>
       <c r="E9" s="11" t="n">
         <v>100</v>
@@ -10488,7 +10488,7 @@
         </is>
       </c>
       <c r="B5" s="7" t="n">
-        <v>588.035</v>
+        <v>615.9059999999999</v>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
@@ -10519,7 +10519,7 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>40d (IS 456:2000)</t>
+          <t>GN table (Fe550, ~50d)</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr"/>
@@ -10531,7 +10531,7 @@
         </is>
       </c>
       <c r="B8" s="8" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="C8" s="8" t="inlineStr">
         <is>
@@ -10546,7 +10546,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>87.51900000000001</v>
+        <v>88.024</v>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
@@ -10561,7 +10561,7 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>51.099</v>
+        <v>50.408</v>
       </c>
       <c r="C10" s="8" t="inlineStr">
         <is>
@@ -10576,7 +10576,7 @@
         </is>
       </c>
       <c r="B11" s="7" t="n">
-        <v>78.79300000000001</v>
+        <v>82.842</v>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
@@ -10591,7 +10591,7 @@
         </is>
       </c>
       <c r="B12" s="9" t="n">
-        <v>246.694</v>
+        <v>262.856</v>
       </c>
       <c r="C12" s="8" t="inlineStr">
         <is>
@@ -10606,7 +10606,7 @@
         </is>
       </c>
       <c r="B13" s="7" t="n">
-        <v>99.73099999999999</v>
+        <v>105.65</v>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
@@ -10621,7 +10621,7 @@
         </is>
       </c>
       <c r="B14" s="9" t="n">
-        <v>24.199</v>
+        <v>26.126</v>
       </c>
       <c r="C14" s="8" t="inlineStr">
         <is>

</xml_diff>